<commit_message>
refactor code to add dataclass
</commit_message>
<xml_diff>
--- a/book_scans.xlsx
+++ b/book_scans.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -459,31 +459,13 @@
           <t>2026-02-16</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>9780140842081</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
+      <c r="B2" t="n">
+        <v>9780140842081</v>
+      </c>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr"/>
+      <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr">
         <is>
           <t>Not Found</t>
@@ -496,10 +478,8 @@
           <t>2026-02-16</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>9780140440485</t>
-        </is>
+      <c r="B3" t="n">
+        <v>9780140440485</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -511,10 +491,8 @@
           <t>Πλάτων</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>1987</t>
-        </is>
+      <c r="E3" t="n">
+        <v>1987</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -533,10 +511,8 @@
           <t>2026-02-16</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>9781845950156</t>
-        </is>
+      <c r="B4" t="n">
+        <v>9781845950156</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -548,10 +524,8 @@
           <t>Василий Семёнович Гроссман, Antony Beevor, Luba Vinogradova</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>2006</t>
-        </is>
+      <c r="E4" t="n">
+        <v>2006</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -559,6 +533,43 @@
         </is>
       </c>
       <c r="G4" t="inlineStr">
+        <is>
+          <t>Found</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-02-16</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>9780340818862</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Watching the English - The Hidden Rules of English Behaviour</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Kate Fox</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>April 11, 2005</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Social life and customs, Nationalcharakter, Volkskultur</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
         <is>
           <t>Found</t>
         </is>

</xml_diff>